<commit_message>
Add 100 / 1k / 10k infra cost comparison tabs to pricing sheet.
Includes mid-high full-stack estimates (Neon, R2, Vercel, Ably, Resend) and scale assumptions.

Co-authored-by: Dralorex <Dralorex@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Rowgon_Pricing_Comparison.xlsx
+++ b/Rowgon_Pricing_Comparison.xlsx
@@ -7,10 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Comparison" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Examples (monthly)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Max Pay" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="How billing works" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Infra Cost 100-10k" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Comparison" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Examples (monthly)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Max Pay" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="How billing works" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Scale Assumptions" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,8 +61,18 @@
       <color rgb="000F766E"/>
       <sz val="12"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00B45309"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00475569"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -85,6 +97,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DBEAFE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1FAE5"/>
       </patternFill>
     </fill>
   </fills>
@@ -114,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -155,6 +182,24 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -520,637 +565,827 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:F44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Rowgon Pricing — Side-by-Side Comparison</t>
+          <t>Rowgon infrastructure cost at scale (hosting stack — not user subscription prices)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Free for personal use. Paid plans = base fee + seats above 5. Yearly = 10× monthly (~2 months free).</t>
+          <t>Stack: Vercel + Neon + Ably + Resend + Cloudflare R2 (+ Stripe % of revenue, separate). Mid-high storage = heavier attachments. Totals are estimates, not quotes.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Seat ladder (all paid plans): 1–5 free · 6–25 = $5/seat · 26–100 = $10/seat · 101+ = $15/seat</t>
-        </is>
-      </c>
-    </row>
-    <row r="4"/>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Feature</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Team</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Business</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Enterprise</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Best for</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>You + friends</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Small teams</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Companies</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Big orgs / many teams</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Base fee (monthly)</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>Google's ~$145/mo figure was Neon+R2 only at 10k. Full stack is higher — especially Ably + Vercel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>MONTHLY TOTALS (full stack)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Users</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Lean / optimized</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Mid-high (typical target)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Heavy / unoptimized</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Mid-high YEARLY</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>What's driving cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>$25–60</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>$40–90</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>$90–180</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="inlineStr">
+        <is>
+          <t>$480–1,080</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>Mostly Vercel Pro + small Neon; R2/Ably still small</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>1,000</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>$80–180</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>$150–320</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>$350–700</t>
+        </is>
+      </c>
+      <c r="E8" s="19" t="inlineStr">
+        <is>
+          <t>$1,800–3,840</t>
+        </is>
+      </c>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>Neon always-on + Ably Standard + Resend digests</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>10,000</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>$220–450</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>$480–1,000</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>$900–1,900+</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="inlineStr">
+        <is>
+          <t>$5,800–12,000</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Ably MAU + Vercel usage + R2 TBs + Neon CU</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>MID-HIGH BREAKDOWN BY SERVICE (monthly $)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>What you pay for</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>100 users</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>1,000 users</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>10,000 users</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Neon (Postgres)</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Compute CU-hrs + DB storage + restore history</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>$5–15</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>$25–60</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>$100–180</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="inlineStr">
+        <is>
+          <t>10k ≈ 1–1.5 CU often-on; text DB ~GB not TB</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Cloudflare R2</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>File storage GB + Class A/B ops (egress $0)</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>$0–5</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>$5–25</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>$55–75</t>
+        </is>
+      </c>
+      <c r="F15" s="14" t="inlineStr">
+        <is>
+          <t>Mid-high @10k ≈ 2–2.5 TB if ~200–250MB/user</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Vercel</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Pro $20 + serverless/CDN overage</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>$20–35</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>$30–70</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>$40–120</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>Unoptimized refreshes/polling push this way up</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Ably</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Realtime chat/badges/presence</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>$0–29</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>$50–150</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>$250–550</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="inlineStr">
+        <is>
+          <t>Biggest sleeper; Free=200 conn only. MAU can dominate</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Resend</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Digests, invites, resets, billing email</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>$0–20</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>$20–35</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>$35–90</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>Free=3k emails/mo; weekly digest scales with users</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Domain / DNS</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>Domain + Cloudflare DNS</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>~$1–2</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>~$1–2</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>~$1–2</t>
+        </is>
+      </c>
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>~$12–20/year domain</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Vercel Cron / jobs</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>Scheduled retention, digests, dunning</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>$0</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>$12 / mo</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>$30 / mo</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>$80 / mo</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Base fee (yearly)</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>$0–10</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>$0–20</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="inlineStr">
+        <is>
+          <t>Cron first; queue product only if jobs get huge</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="40" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>WorkOS SSO</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>Enterprise SSO only</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>$0</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>$120 / yr</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>$300 / yr</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>$800 / yr</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Who pays</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Nobody</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>That workspace</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>That workspace</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>Whole organization</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>People (seats)</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Up to 5</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Up to 25</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Up to 100</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>As many as you type</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Extra seat cost</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>$5 each after 5</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>$5 then $10 after 25</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>Same + $15 after 100</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Workspaces</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>1 free</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Upgrade + free slot again</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Same</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Unlimited under company</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Custom roles</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>Unlimited</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>Unlimited</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Tasks / claim / review</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>Friends &amp; DMs</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Group chats</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Unlimited</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Unlimited</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>Unlimited</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Data retention</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>90 days</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>1 year</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>Company sets rules</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>File storage</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>5 GB</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>50 GB</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>Shared company pool</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="28" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Export / backup</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>Basic</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>Full</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>Full</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Audit log</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>Yes (whole company)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Admin tools (bulk invite, etc.)</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>$0</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="28" customHeight="1">
+          <t>$0–low</t>
+        </is>
+      </c>
+      <c r="F21" s="14" t="inlineStr">
+        <is>
+          <t>Not needed for raw user count; Enterprise feature</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="40" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Calendar sync (Google etc.)</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Virus scan</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>Deferred</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$0</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>$0</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="28" customHeight="1">
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
+        <is>
+          <t>Add later when uploads are untrusted/heavy</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="40" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Company login (SSO)</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>% of revenue (not per user)</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>varies</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>varies</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Yes (when ready)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>Support</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Docs</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>Priority email</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>Named person + SLA</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="28" customHeight="1">
+          <t>varies</t>
+        </is>
+      </c>
+      <c r="F23" s="14" t="inlineStr">
+        <is>
+          <t>~2.9%+$0.30 + Billing % — not hosting</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="40" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>MID-HIGH TOTAL (infra)</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Sum of hosting stack (excl. Stripe)</t>
+        </is>
+      </c>
+      <c r="C24" s="19" t="inlineStr">
+        <is>
+          <t>$40–90</t>
+        </is>
+      </c>
+      <c r="D24" s="19" t="inlineStr">
+        <is>
+          <t>$150–320</t>
+        </is>
+      </c>
+      <c r="E24" s="19" t="inlineStr">
+        <is>
+          <t>$480–1,000</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Use middle of range for planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="40" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>MAX PAY / MONTH (at plan seat cap)</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>$112</t>
-        </is>
-      </c>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>$880</t>
-        </is>
-      </c>
-      <c r="E25" s="8" t="inlineStr">
-        <is>
-          <t>No fixed max — scales with seats</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>MAX PAY / YEAR (≈10× monthly)</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="inlineStr">
-        <is>
-          <t>$1,120</t>
-        </is>
-      </c>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>$8,800</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>No fixed max — scales with seats</t>
+          <t>MID-HIGH YEARLY</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>×12</t>
+        </is>
+      </c>
+      <c r="C25" s="19" t="inlineStr">
+        <is>
+          <t>$480–1,080</t>
+        </is>
+      </c>
+      <c r="D25" s="19" t="inlineStr">
+        <is>
+          <t>$1,800–3,840</t>
+        </is>
+      </c>
+      <c r="E25" s="19" t="inlineStr">
+        <is>
+          <t>$5,800–12,000</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>Round planning numbers</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>GOOGLE'S 10k NUMBER VS FULL STACK</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Slice</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Yearly</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="32" customHeight="1">
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t>Google: Neon + R2 only (their math)</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="inlineStr">
+        <is>
+          <t>~$145</t>
+        </is>
+      </c>
+      <c r="C30" s="20" t="inlineStr">
+        <is>
+          <t>~$1,740</t>
+        </is>
+      </c>
+      <c r="D30" s="20" t="inlineStr">
+        <is>
+          <t>OK ballpark for DB+files at 2.5TB — incomplete for Rowgon</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="32" customHeight="1">
+      <c r="A31" s="21" t="inlineStr">
+        <is>
+          <t>Full mid-high stack (this sheet)</t>
+        </is>
+      </c>
+      <c r="B31" s="21" t="inlineStr">
+        <is>
+          <t>~$480–1,000</t>
+        </is>
+      </c>
+      <c r="C31" s="21" t="inlineStr">
+        <is>
+          <t>~$5,800–12,000</t>
+        </is>
+      </c>
+      <c r="D31" s="21" t="inlineStr">
+        <is>
+          <t>Includes Vercel + Ably + Resend</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="32" customHeight="1">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>Ably alone if all 10k are MAU @ ~$0.05</t>
+        </is>
+      </c>
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>~$500 (+$29 base)</t>
+        </is>
+      </c>
+      <c r="C32" s="13" t="inlineStr">
+        <is>
+          <t>~$6,300</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="inlineStr">
+        <is>
+          <t>Why Google total is too low</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>STORAGE ASSUMPTIONS USED</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Users</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Neon DB data (text)</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>R2 files (mid-high)</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>R2 storage $ (approx)</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="36" customHeight="1">
+      <c r="A37" s="17" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>0.2–1 GB</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>10–50 GB</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>$0–1 (near free tier)</t>
+        </is>
+      </c>
+      <c r="E37" s="13" t="inlineStr">
+        <is>
+          <t>Often still in R2 free 10GB if careful</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="36" customHeight="1">
+      <c r="A38" s="17" t="inlineStr">
+        <is>
+          <t>1,000</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>1–5 GB</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>100–400 GB</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>$1.5–6</t>
+        </is>
+      </c>
+      <c r="E38" s="13" t="inlineStr">
+        <is>
+          <t>~100–400MB/user average attachments</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="36" customHeight="1">
+      <c r="A39" s="17" t="inlineStr">
+        <is>
+          <t>10,000</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>10–25 GB</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>2.0–2.5 TB</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>~$30–37 storage + ops ≈ $55–75</t>
+        </is>
+      </c>
+      <c r="E39" s="13" t="inlineStr">
+        <is>
+          <t>~200–250MB/user — Google mid-high case</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="22" t="inlineStr">
+        <is>
+          <t>R2 does NOT compound: storing 12GB unused stays ~12GB next month (pay each month for what's still there), not 24GB.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="22" t="inlineStr">
+        <is>
+          <t>Revenue note (not hosting): Stripe fees are a % of money collected. User subscription prices are on other tabs (Free/Team/Business/Enterprise).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A3:E3"/>
+  <mergeCells count="5">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:F3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1162,8 +1397,649 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Rowgon Pricing — Side-by-Side Comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Free for personal use. Paid plans = base fee + seats above 5. Yearly = 10× monthly (~2 months free).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Seat ladder (all paid plans): 1–5 free · 6–25 = $5/seat · 26–100 = $10/seat · 101+ = $15/seat</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Best for</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>You + friends</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Small teams</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Companies</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Big orgs / many teams</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Base fee (monthly)</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>$12 / mo</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>$30 / mo</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>$80 / mo</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Base fee (yearly)</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>$120 / yr</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>$300 / yr</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>$800 / yr</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Who pays</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Nobody</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>That workspace</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>That workspace</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Whole organization</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>People (seats)</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Up to 5</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Up to 25</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Up to 100</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>As many as you type</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Extra seat cost</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>$5 each after 5</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>$5 then $10 after 25</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Same + $15 after 100</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Workspaces</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>1 free</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Upgrade + free slot again</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Unlimited under company</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Custom roles</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Unlimited</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Unlimited</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Tasks / claim / review</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Friends &amp; DMs</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Group chats</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Unlimited</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Unlimited</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Unlimited</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Data retention</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>90 days</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>1 year</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>3 years</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Company sets rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>File storage</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>5 GB</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>50 GB</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Shared company pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Export / backup</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Audit log</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Yes (whole company)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Admin tools (bulk invite, etc.)</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Calendar sync (Google etc.)</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Company login (SSO)</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>Yes (when ready)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Priority email</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Named person + SLA</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>MAX PAY / MONTH (at plan seat cap)</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>$112</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>$880</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>No fixed max — scales with seats</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>MAX PAY / YEAR (≈10× monthly)</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>$1,120</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>$8,800</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>No fixed max — scales with seats</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A3:E3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -1186,7 +2062,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1389,8 +2264,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
@@ -1412,7 +2285,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
@@ -1427,7 +2299,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
@@ -1454,14 +2325,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -1738,14 +2609,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="88" customWidth="1" min="2" max="2"/>
@@ -1966,4 +2837,164 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>How to read the scale cost ranges</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="23" t="inlineStr">
+        <is>
+          <t>Lean / optimized</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Optimistic UI, few full-page refreshes, Ably payloads small, attachment caps, digests opt-in, Neon not oversized</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>Mid-high (target planning)</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Serious daily use + mid-high attachments; Ably on for many actives; Pro hosting; weekly digests</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="23" t="inlineStr">
+        <is>
+          <t>Heavy / unoptimized</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Current-style full RSC refresh on chat, heavy polling, fat Ably MAU, large unchecked uploads, always-on big Neon</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>100 users</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Still mostly small-bill territory; Vercel Pro may already be wanted for commercial use</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>1,000 users</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Free tiers of Ably/Resend/Neon usually exceeded; treat as paid SaaS ops</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>10,000 users</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Real commercial infra; Ably + Vercel usage often exceed Neon+R2 combined</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>Not included in totals</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Your time, support staff, Apple/Google fees, ads, legal, virus scan, WorkOS at scale, Stripe processing fees</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t>Neon rate basis</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>~$0.106/CU-hour Launch; 1 CU always-on ≈ $77/mo compute before storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="23" t="inlineStr">
+        <is>
+          <t>R2 rate basis</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>$0.015/GB-mo; Class A $4.50/M; Class B $0.36/M; 10GB + ops free; egress $0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>Ably watch-out</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Free = 200 concurrent connections. Standard from ~$29 + usage/MAU — can dwarf storage at 10k</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>